<commit_message>
Refresh notebook outputs and reorganize model artifacts
</commit_message>
<xml_diff>
--- a/app/data/raw/lotto_history_latest.xlsx
+++ b/app/data/raw/lotto_history_latest.xlsx
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1217"/>
+  <dimension ref="A1:L1218"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7.70703125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -54072,6 +54072,50 @@
         </is>
       </c>
     </row>
+    <row r="1218">
+      <c r="A1218" t="n">
+        <v>1217</v>
+      </c>
+      <c r="B1218" t="n">
+        <v>1217</v>
+      </c>
+      <c r="C1218" t="n">
+        <v>8</v>
+      </c>
+      <c r="D1218" t="n">
+        <v>10</v>
+      </c>
+      <c r="E1218" t="n">
+        <v>15</v>
+      </c>
+      <c r="F1218" t="n">
+        <v>20</v>
+      </c>
+      <c r="G1218" t="n">
+        <v>29</v>
+      </c>
+      <c r="H1218" t="n">
+        <v>31</v>
+      </c>
+      <c r="I1218" t="n">
+        <v>41</v>
+      </c>
+      <c r="J1218" t="inlineStr">
+        <is>
+          <t>1등</t>
+        </is>
+      </c>
+      <c r="K1218" t="inlineStr">
+        <is>
+          <t>14 명</t>
+        </is>
+      </c>
+      <c r="L1218" t="inlineStr">
+        <is>
+          <t>2,179,738,018 원</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>